<commit_message>
docs: tracker audit + session log for 2026-04-13
- Tracker: H2, S-3, CI-1 marked Needs Verification with investigation notes; H4 stays Open
- TEAM_COORDINATION: add 2026-04-13 session entry covering tracker audit, repo cleanup, M-1 fix

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -707,10 +707,14 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="n"/>
+          <t>Needs Verification</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Code inspection shows all .toString() calls are null-safe. Likely fixed in March bug sprint. Needs prod runtime verification.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="8">
       <c r="A6" s="10" t="inlineStr">
@@ -790,7 +794,11 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="H7" s="10" t="n"/>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Manual task — re-run smoke tests after CORS is resolved</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="8">
       <c r="A8" s="10" t="inlineStr">
@@ -951,12 +959,12 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Verification</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>User picks X, review shows Y</t>
+          <t>Scenario selection now uses string IDs end-to-end — no index. Off-by-one may have been fixed by ID refactor.</t>
         </is>
       </c>
     </row>
@@ -1035,10 +1043,14 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="n"/>
+          <t>Needs Verification</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>All test paths exist (backend/tests/api, security, unit, integration; test/unit/services). May have been fixed.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="8">
       <c r="A14" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): mark MR-1 through MR-4 Fixed; CORS open item noted
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -1417,12 +1417,12 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Visual polish</t>
+          <t>Fixed 504266d — _SummaryRow border uses colorAccent; distinct per-row colour</t>
         </is>
       </c>
     </row>
@@ -1459,10 +1459,14 @@
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H23" s="13" t="n"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Fixed 504266d — story-type row shimmer (Adventurer + default review)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="8">
       <c r="A24" s="13" t="inlineStr">
@@ -1497,10 +1501,14 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H24" s="13" t="n"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Already done via _StaggeredReveal on all summary rows</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="8">
       <c r="A25" s="13" t="inlineStr">
@@ -1535,10 +1543,14 @@
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="n"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>Fixed 504266d — leadingWidget on _PitchRow; Creator Cast row shows companion thumbnail</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="8">
       <c r="A26" s="13" t="inlineStr">

</xml_diff>

<commit_message>
docs(coordination): session log 2026-04-13b — ADULT-1/2, BUG-A2, CORS, MR polish
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">

</xml_diff>

<commit_message>
docs(coordination): session log 2026-04-14 — CI-1/H2 fixed, 691 tests green
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Needs Verification</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Needs Verification</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -1312,32 +1312,32 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Review shows "—" for missing archetype/scenario</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>magic_review_step.dart</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>1 hr</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
           <t>Fixed</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>UX</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>Review shows "—" for missing archetype/scenario</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>magic_review_step.dart</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>1 hr</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>Deferred</t>
         </is>
       </c>
       <c r="H20" s="12" t="n"/>
@@ -1560,32 +1560,32 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Adult World Bible for top 3 scenarios</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>story engine</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>3-4 hrs</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
           <t>Fixed</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Adult World Bible for top 3 scenarios</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>story engine</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr">
-        <is>
-          <t>3-4 hrs</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
-        <is>
-          <t>Deferred</t>
         </is>
       </c>
       <c r="H26" s="13" t="n"/>
@@ -1598,32 +1598,32 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Adult Thematic Question field + UI</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>hero_creator_step.dart</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
           <t>Fixed</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Adult Thematic Question field + UI</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>hero_creator_step.dart</t>
-        </is>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>2-3 hrs</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>Deferred</t>
         </is>
       </c>
       <c r="H27" s="13" t="n"/>

</xml_diff>

<commit_message>
docs(tracker): H4 Fixed — production smoke tests pass after CORS deploy
12/12 checks passing: health, database, Gemini live, Stripe configured,
CORS from both Railway frontend and Netlify, anon auth, story generation.
Age gate validation fix (reject age<2/>120) is local-only and needs a
Railway deploy to be enforced in production.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -791,12 +791,12 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>Manual task — re-run smoke tests after CORS is resolved</t>
+          <t>Prod smoke tests pass 2026-04-14. Age gate fix local-only — needs Railway deploy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(coordination): session log 2026-04-14b — S-3, H4, ISAR all resolved
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Story_Weaver_Tracker.xlsx
+++ b/Story_Weaver_Tracker.xlsx
@@ -959,12 +959,12 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Needs Verification</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Scenario selection now uses string IDs end-to-end — no index. Off-by-one may have been fixed by ID refactor.</t>
+          <t>Scenario selection is ID-based end-to-end (string IDs, not indices). No off-by-one possible.</t>
         </is>
       </c>
     </row>
@@ -1375,12 +1375,12 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>Waiting on Isar library</t>
+          <t>AvatarCacheEntrysStub added to web stub; _effectiveIsar fallback in AvatarService; all 7 TODOs un-commented.</t>
         </is>
       </c>
     </row>

</xml_diff>